<commit_message>
Align fund type classification with EID platform categories
Update classify_product_type to use the nine official fund types from
eid.csrc.gov.cn (股票型, 货币型, 债券型, 混合型, QDII, 短期理财债券型,
基金中基金 (FOF), 商品基金, 不动产投资信托基金). Add normalize_fund_type
to map legacy website labels (指数型, ETF联接基金, etc.) and regenerate Excel.

Co-authored-by: linzhuoran79 <linzhuoran79@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/outputs/fund_records/易方达_广发_2025_2026Q1_报会与首发记录.xlsx
+++ b/outputs/fund_records/易方达_广发_2025_2026Q1_报会与首发记录.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -482,10 +482,22 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>产品类型口径</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>与证监会基金电子披露平台（eid.csrc.gov.cn）“基金类型”下拉选项一致：股票型、货币型、债券型、混合型、QDII、短期理财债券型、基金中基金 (FOF)、商品基金、不动产投资信托基金。</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
           <t>注意</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>托管人为证券公司的ETF/联接基金保留“托管人”原文；字段名写作“托管行/托管人”。</t>
         </is>
@@ -648,7 +660,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>债券型/固收</t>
+          <t>短期理财债券型</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -707,7 +719,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -770,7 +782,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -888,7 +900,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>债券型/固收</t>
+          <t>债券型</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -1073,7 +1085,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>债券型/固收</t>
+          <t>短期理财债券型</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1195,7 +1207,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>债券型/固收</t>
+          <t>债券型</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1254,7 +1266,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1313,7 +1325,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1376,7 +1388,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>债券型/固收</t>
+          <t>债券型</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1435,7 +1447,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>债券型/固收</t>
+          <t>债券型</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1494,7 +1506,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1557,7 +1569,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1620,7 +1632,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1746,7 +1758,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>债券型/固收</t>
+          <t>债券型</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1809,7 +1821,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>FOF</t>
+          <t>基金中基金 (FOF)</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1872,7 +1884,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1935,7 +1947,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1998,7 +2010,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -2124,7 +2136,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -2187,7 +2199,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -2250,7 +2262,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -2313,7 +2325,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -2376,7 +2388,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -2565,7 +2577,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -2801,7 +2813,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -2864,7 +2876,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -2990,7 +3002,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -3045,7 +3057,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -3222,7 +3234,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -3285,7 +3297,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -3340,7 +3352,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -3450,7 +3462,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -3513,7 +3525,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -3639,7 +3651,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>债券型/固收</t>
+          <t>债券型</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -3926,7 +3938,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -3989,7 +4001,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -4107,7 +4119,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -4162,7 +4174,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -4221,7 +4233,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -4280,7 +4292,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -4335,7 +4347,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -4453,7 +4465,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>FOF</t>
+          <t>基金中基金 (FOF)</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -4579,7 +4591,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -4634,7 +4646,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>纯债/债券型</t>
+          <t>债券型</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -4693,7 +4705,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>FOF</t>
+          <t>基金中基金 (FOF)</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -4756,7 +4768,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>FOF</t>
+          <t>基金中基金 (FOF)</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -4819,7 +4831,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -4929,7 +4941,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -4984,7 +4996,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -5110,7 +5122,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -5165,7 +5177,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -5220,7 +5232,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>FOF</t>
+          <t>基金中基金 (FOF)</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -5346,7 +5358,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>FOF</t>
+          <t>基金中基金 (FOF)</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -5409,7 +5421,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -5464,7 +5476,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -5527,7 +5539,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -5653,7 +5665,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -5708,7 +5720,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -5763,7 +5775,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -5826,7 +5838,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -6015,7 +6027,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>债券型/固收</t>
+          <t>债券型</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -6078,7 +6090,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -6133,7 +6145,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -6188,7 +6200,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -6243,7 +6255,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -6306,7 +6318,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>FOF</t>
+          <t>基金中基金 (FOF)</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -6369,7 +6381,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -6491,7 +6503,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -6554,7 +6566,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -6617,7 +6629,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -6743,7 +6755,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -6798,7 +6810,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -6857,7 +6869,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -7034,7 +7046,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
@@ -7089,7 +7101,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -7152,7 +7164,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -7215,7 +7227,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>债券型/固收</t>
+          <t>债券型</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
@@ -7274,7 +7286,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
@@ -7337,7 +7349,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -7400,7 +7412,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -7463,7 +7475,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -7526,7 +7538,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -7589,7 +7601,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>债券型/固收</t>
+          <t>债券型</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -7648,7 +7660,7 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>债券型/固收</t>
+          <t>债券型</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
@@ -7707,7 +7719,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>债券型/固收</t>
+          <t>债券型</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -7770,7 +7782,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
@@ -7833,7 +7845,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
@@ -7959,7 +7971,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
@@ -8022,7 +8034,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
@@ -8085,7 +8097,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
@@ -8148,7 +8160,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
@@ -8211,7 +8223,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
@@ -8274,7 +8286,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
@@ -8400,7 +8412,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
@@ -8463,7 +8475,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
@@ -8526,7 +8538,7 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
@@ -8589,7 +8601,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>债券型/固收</t>
+          <t>债券型</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
@@ -8652,7 +8664,7 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
@@ -8715,7 +8727,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
@@ -8778,7 +8790,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
@@ -8841,7 +8853,7 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
@@ -8967,7 +8979,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
@@ -9030,7 +9042,7 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
@@ -9093,7 +9105,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>FOF</t>
+          <t>基金中基金 (FOF)</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
@@ -9156,7 +9168,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
@@ -9219,7 +9231,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
@@ -9282,7 +9294,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>FOF</t>
+          <t>基金中基金 (FOF)</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
@@ -9345,7 +9357,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
@@ -9408,7 +9420,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
@@ -9471,7 +9483,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
@@ -9597,7 +9609,7 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
@@ -9656,7 +9668,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
@@ -10089,7 +10101,7 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>商品基金</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
@@ -10144,7 +10156,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
@@ -10266,7 +10278,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
@@ -10384,7 +10396,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D163" t="inlineStr">
@@ -10447,7 +10459,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D164" t="inlineStr">
@@ -10510,7 +10522,7 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D165" t="inlineStr">
@@ -10573,7 +10585,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>QDII</t>
         </is>
       </c>
       <c r="D166" t="inlineStr">
@@ -10636,7 +10648,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>FOF</t>
+          <t>基金中基金 (FOF)</t>
         </is>
       </c>
       <c r="D167" t="inlineStr">
@@ -10880,7 +10892,7 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D171" t="inlineStr">
@@ -11061,7 +11073,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D174" t="inlineStr">
@@ -11124,7 +11136,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>FOF</t>
+          <t>基金中基金 (FOF)</t>
         </is>
       </c>
       <c r="D175" t="inlineStr">
@@ -11187,7 +11199,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D176" t="inlineStr">
@@ -11242,7 +11254,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D177" t="inlineStr">
@@ -11305,7 +11317,7 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D178" t="inlineStr">
@@ -11360,7 +11372,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D179" t="inlineStr">
@@ -11423,7 +11435,7 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D180" t="inlineStr">
@@ -11478,7 +11490,7 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D181" t="inlineStr">
@@ -11541,7 +11553,7 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D182" t="inlineStr">
@@ -11600,7 +11612,7 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D183" t="inlineStr">
@@ -11655,7 +11667,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D184" t="inlineStr">
@@ -11714,7 +11726,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D185" t="inlineStr">
@@ -11773,7 +11785,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D186" t="inlineStr">
@@ -11828,7 +11840,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D187" t="inlineStr">
@@ -12009,7 +12021,7 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D190" t="inlineStr">
@@ -12064,7 +12076,7 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D191" t="inlineStr">
@@ -12127,7 +12139,7 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>FOF</t>
+          <t>基金中基金 (FOF)</t>
         </is>
       </c>
       <c r="D192" t="inlineStr">
@@ -12253,7 +12265,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D194" t="inlineStr">
@@ -12308,7 +12320,7 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D195" t="inlineStr">
@@ -12363,7 +12375,7 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D196" t="inlineStr">
@@ -12426,7 +12438,7 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D197" t="inlineStr">
@@ -12481,7 +12493,7 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D198" t="inlineStr">
@@ -12536,7 +12548,7 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D199" t="inlineStr">
@@ -12599,7 +12611,7 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D200" t="inlineStr">
@@ -12662,7 +12674,7 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D201" t="inlineStr">
@@ -12717,7 +12729,7 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>FOF</t>
+          <t>基金中基金 (FOF)</t>
         </is>
       </c>
       <c r="D202" t="inlineStr">
@@ -12780,7 +12792,7 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D203" t="inlineStr">
@@ -12843,7 +12855,7 @@
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D204" t="inlineStr">
@@ -12906,7 +12918,7 @@
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D205" t="inlineStr">
@@ -12961,7 +12973,7 @@
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D206" t="inlineStr">
@@ -13024,7 +13036,7 @@
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>FOF</t>
+          <t>基金中基金 (FOF)</t>
         </is>
       </c>
       <c r="D207" t="inlineStr">
@@ -13087,7 +13099,7 @@
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D208" t="inlineStr">
@@ -13150,7 +13162,7 @@
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D209" t="inlineStr">
@@ -13213,7 +13225,7 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D210" t="inlineStr">
@@ -13268,7 +13280,7 @@
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D211" t="inlineStr">
@@ -13386,7 +13398,7 @@
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D213" t="inlineStr">
@@ -13508,7 +13520,7 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D215" t="inlineStr">
@@ -13571,7 +13583,7 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>债券型/固收</t>
+          <t>债券型</t>
         </is>
       </c>
       <c r="D216" t="inlineStr">
@@ -13626,7 +13638,7 @@
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D217" t="inlineStr">
@@ -13689,7 +13701,7 @@
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D218" t="inlineStr">
@@ -13752,7 +13764,7 @@
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D219" t="inlineStr">
@@ -13815,7 +13827,7 @@
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>FOF</t>
+          <t>基金中基金 (FOF)</t>
         </is>
       </c>
       <c r="D220" t="inlineStr">
@@ -13937,7 +13949,7 @@
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D222" t="inlineStr">
@@ -14000,7 +14012,7 @@
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>债券型/固收</t>
+          <t>债券型</t>
         </is>
       </c>
       <c r="D223" t="inlineStr">
@@ -14063,7 +14075,7 @@
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>FOF</t>
+          <t>基金中基金 (FOF)</t>
         </is>
       </c>
       <c r="D224" t="inlineStr">
@@ -14126,7 +14138,7 @@
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D225" t="inlineStr">
@@ -14189,7 +14201,7 @@
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D226" t="inlineStr">
@@ -14244,7 +14256,7 @@
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D227" t="inlineStr">
@@ -14307,7 +14319,7 @@
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D228" t="inlineStr">
@@ -14370,7 +14382,7 @@
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D229" t="inlineStr">
@@ -14433,7 +14445,7 @@
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D230" t="inlineStr">
@@ -14496,7 +14508,7 @@
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D231" t="inlineStr">
@@ -14555,7 +14567,7 @@
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D232" t="inlineStr">
@@ -14618,7 +14630,7 @@
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D233" t="inlineStr">
@@ -14677,7 +14689,7 @@
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D234" t="inlineStr">
@@ -14736,7 +14748,7 @@
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>指数型/ETF/联接</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="D235" t="inlineStr">
@@ -14964,7 +14976,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>指数型</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -15374,7 +15386,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>指数型</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -15456,7 +15468,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>指数型</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -15620,7 +15632,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>指数型</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -15784,7 +15796,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>指数型</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -15866,7 +15878,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>指数型</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -16030,7 +16042,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>指数型</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -16112,7 +16124,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>指数型</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -16194,7 +16206,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>指数型</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -16276,7 +16288,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>指数型</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -16358,7 +16370,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>FOF</t>
+          <t>基金中基金 (FOF)</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -16522,7 +16534,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>指数型</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -16604,7 +16616,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>指数型</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -16768,7 +16780,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>指数型</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -16932,7 +16944,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>指数型</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -17014,7 +17026,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>指数型</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -17178,7 +17190,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>指数型</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -17260,7 +17272,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>指数型</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -17342,7 +17354,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>FOF</t>
+          <t>基金中基金 (FOF)</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -17588,7 +17600,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>指数型</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -17670,7 +17682,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>指数型</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -17916,7 +17928,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>指数型</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -18080,7 +18092,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>FOF</t>
+          <t>基金中基金 (FOF)</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -18162,7 +18174,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>FOF</t>
+          <t>基金中基金 (FOF)</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -18326,7 +18338,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>指数型</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -18408,7 +18420,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>指数型</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -18572,7 +18584,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>ETF联接基金</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -18818,7 +18830,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>ETF联接基金</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -18982,7 +18994,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>ETF联接基金</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -19310,7 +19322,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>ETF联接基金</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -19966,7 +19978,7 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>ETF联接基金</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -20130,7 +20142,7 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>基金中基金</t>
+          <t>基金中基金 (FOF)</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -20458,7 +20470,7 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>ETF联接基金</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
@@ -21114,7 +21126,7 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>ETF联接基金</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -21442,7 +21454,7 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>ETF联接基金</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -21688,7 +21700,7 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>ETF联接基金</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
@@ -21770,7 +21782,7 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>ETF联接基金</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
@@ -22180,7 +22192,7 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>ETF联接基金</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
@@ -22508,7 +22520,7 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>基金中基金</t>
+          <t>基金中基金 (FOF)</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
@@ -22836,7 +22848,7 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>ETF联接基金</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
@@ -22918,7 +22930,7 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>ETF联接基金</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
@@ -23246,7 +23258,7 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>基金中基金</t>
+          <t>基金中基金 (FOF)</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
@@ -23820,7 +23832,7 @@
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>ETF联接基金</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="F110" t="inlineStr">
@@ -24148,7 +24160,7 @@
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>ETF联接基金</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="F114" t="inlineStr">
@@ -25050,7 +25062,7 @@
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>基金中基金</t>
+          <t>基金中基金 (FOF)</t>
         </is>
       </c>
       <c r="F125" t="inlineStr">
@@ -25132,7 +25144,7 @@
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>ETF联接基金</t>
+          <t>股票型</t>
         </is>
       </c>
       <c r="F126" t="inlineStr">

</xml_diff>

<commit_message>
Map infrastructure and real-estate funds to REIT EID type
Co-authored-by: linzhuoran79 <linzhuoran79@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/outputs/fund_records/易方达_广发_2025_2026Q1_报会与首发记录.xlsx
+++ b/outputs/fund_records/易方达_广发_2025_2026Q1_报会与首发记录.xlsx
@@ -6444,7 +6444,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>未识别</t>
+          <t>不动产投资信托基金</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -10829,7 +10829,7 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>未识别</t>
+          <t>不动产投资信托基金</t>
         </is>
       </c>
       <c r="D170" t="inlineStr">

</xml_diff>